<commit_message>
Add comprehensive synthetic empaTAPP example exercising all schema properties
exampleempaTAPP-all.json is hand-authored alongside the 10 publication-derived
P1..P10 examples. It populates every property allowed by tappDefinition + the
empaTAPP overlay (4 EMPA top-level props, 6 methodParameters, 14-column
analyteTemplate with default analyte rows, full instrument hierarchy,
geosparql-qualified location, agent, HowTo workflow, quality measurements,
related links, funding) and serves as a structural reference for new authors.
README and AGENTS.md updated to describe it; AGENTS.md also captures the
authoring gotchas surfaced during validation iteration (inDefinedTermSet
shape, geosparql object form, schema:relatedLink as CreativeWork, etc.).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TAPP_EPMA_filled.xlsx
+++ b/docs/TAPP_EPMA_filled.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/944a82e2ddcde9eb/Documents/GithubC/USGIN/geochemBuildingBlocks/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="278" documentId="11_3C209AD99577444EEF615C96566D1EBF266D99FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{587812C6-6FFF-49C7-9FA9-EF533DB21C2F}"/>
+  <xr:revisionPtr revIDLastSave="279" documentId="11_3C209AD99577444EEF615C96566D1EBF266D99FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88AEFEA8-2993-49E2-8699-4CC11906C290}"/>
   <bookViews>
-    <workbookView xWindow="555" yWindow="690" windowWidth="27930" windowHeight="14610" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1065" windowWidth="27930" windowHeight="14610" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TAPP" sheetId="1" r:id="rId1"/>
@@ -2109,7 +2109,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="182">
+  <cellXfs count="181">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2619,9 +2619,6 @@
     <xf numFmtId="0" fontId="6" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2706,6 +2703,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2894,9 +2895,9 @@
     <col min="5" max="5" width="32" style="32" customWidth="1"/>
     <col min="6" max="6" width="7.85546875" style="4" customWidth="1"/>
     <col min="7" max="7" width="17.140625" style="4" customWidth="1"/>
-    <col min="8" max="8" width="38" style="167" customWidth="1"/>
-    <col min="9" max="12" width="38" style="58" customWidth="1"/>
-    <col min="13" max="17" width="30" style="58" customWidth="1"/>
+    <col min="8" max="8" width="38" style="167" hidden="1" customWidth="1"/>
+    <col min="9" max="12" width="38" style="58" hidden="1" customWidth="1"/>
+    <col min="13" max="17" width="30" style="58" hidden="1" customWidth="1"/>
     <col min="18" max="18" width="8.42578125" style="168" customWidth="1"/>
     <col min="19" max="19" width="37.140625" style="4" customWidth="1"/>
     <col min="20" max="20" width="49.140625" style="4" customWidth="1"/>
@@ -5234,7 +5235,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="S51" s="181" t="s">
+      <c r="S51" s="3" t="s">
         <v>213</v>
       </c>
       <c r="T51" s="3" t="s">
@@ -5278,7 +5279,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="S52" s="181" t="s">
+      <c r="S52" s="3" t="s">
         <v>213</v>
       </c>
       <c r="T52" s="3" t="s">
@@ -5322,7 +5323,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="S53" s="181" t="s">
+      <c r="S53" s="3" t="s">
         <v>213</v>
       </c>
       <c r="T53" s="3" t="s">
@@ -5412,7 +5413,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="S55" s="181" t="s">
+      <c r="S55" s="3" t="s">
         <v>213</v>
       </c>
       <c r="T55" s="3" t="s">
@@ -5456,7 +5457,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="S56" s="181" t="s">
+      <c r="S56" s="3" t="s">
         <v>213</v>
       </c>
       <c r="T56" s="3" t="s">
@@ -5566,7 +5567,7 @@
         <f t="shared" ref="R59:R68" si="4">COUNTA(H59:Q59)/10</f>
         <v>0.9</v>
       </c>
-      <c r="S59" s="181" t="s">
+      <c r="S59" s="3" t="s">
         <v>213</v>
       </c>
       <c r="T59" s="3" t="s">
@@ -5616,7 +5617,7 @@
         <f t="shared" si="4"/>
         <v>0.3</v>
       </c>
-      <c r="S60" s="181" t="s">
+      <c r="S60" s="3" t="s">
         <v>213</v>
       </c>
       <c r="T60" s="3" t="s">
@@ -5660,7 +5661,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="S61" s="181" t="s">
+      <c r="S61" s="3" t="s">
         <v>213</v>
       </c>
       <c r="T61" s="3" t="s">
@@ -5748,7 +5749,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="S63" s="181" t="s">
+      <c r="S63" s="3" t="s">
         <v>213</v>
       </c>
       <c r="T63" s="3" t="s">
@@ -5802,7 +5803,7 @@
         <f t="shared" si="4"/>
         <v>0.5</v>
       </c>
-      <c r="S64" s="181" t="s">
+      <c r="S64" s="3" t="s">
         <v>213</v>
       </c>
       <c r="T64" s="3" t="s">
@@ -5846,7 +5847,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="S65" s="181" t="s">
+      <c r="S65" s="3" t="s">
         <v>213</v>
       </c>
       <c r="T65" s="3"/>
@@ -5888,7 +5889,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="S66" s="181" t="s">
+      <c r="S66" s="3" t="s">
         <v>213</v>
       </c>
       <c r="T66" s="3" t="s">
@@ -5932,7 +5933,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="S67" s="181" t="s">
+      <c r="S67" s="3" t="s">
         <v>213</v>
       </c>
       <c r="T67" s="9" t="s">
@@ -5976,7 +5977,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="S68" s="181" t="s">
+      <c r="S68" s="3" t="s">
         <v>213</v>
       </c>
       <c r="T68" s="9" t="s">

</xml_diff>

<commit_message>
Fix TAPP_EPMA impl-notes typos and regenerate empaTAPP examples
Repairs three impl-notes errors in the "Default Accelerating Voltage"
row of the TAPP worksheet (extra colon after `property:`, missing colon
after `readonly`, stray `parameter:` prefix before `readOnly`) that were
producing duplicate methodParameters entries with valueName "readOnly"
and silently dropping the property-track tag. Regenerates all ten
per-publication empaTAPP examples and the empaTAPP schema.yaml from
the corrected spreadsheet; the schema now correctly emits a top-level
ada:acceleratingVoltageDefault property alongside the existing
beamDiameterDefault and beamCurrentDefault.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TAPP_EPMA_filled.xlsx
+++ b/docs/TAPP_EPMA_filled.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/944a82e2ddcde9eb/Documents/GithubC/USGIN/geochemBuildingBlocks/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="279" documentId="11_3C209AD99577444EEF615C96566D1EBF266D99FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88AEFEA8-2993-49E2-8699-4CC11906C290}"/>
+  <xr:revisionPtr revIDLastSave="299" documentId="11_3C209AD99577444EEF615C96566D1EBF266D99FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F1E778BF-00DE-4010-B5A4-4CECD611067F}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1065" windowWidth="27930" windowHeight="14610" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8520" yWindow="990" windowWidth="27930" windowHeight="14610" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TAPP" sheetId="1" r:id="rId1"/>
@@ -91,7 +91,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="681" uniqueCount="461">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="681" uniqueCount="463">
   <si>
     <t>Metadata Item</t>
   </si>
@@ -340,9 +340,6 @@
     <t>Silicate minerals (tissintite, maskelynite, pigeonite, fayalite)</t>
   </si>
   <si>
-    <t>Maskelynite, melt inclusion glasses, silica glass, coesite aggregates, mesostasis</t>
-  </si>
-  <si>
     <t>Olivine, pyroxene, Fe-Ti-Cr oxides, maskelynite, phosphate, sulfide, glass</t>
   </si>
   <si>
@@ -706,28 +703,16 @@
     <t>e.g., 10 | 50 | 100</t>
   </si>
   <si>
-    <t>Element specific</t>
-  </si>
-  <si>
     <t>5</t>
   </si>
   <si>
     <t>10</t>
   </si>
   <si>
-    <t>20 nA (silicates/oxides); 10 nA (glass/maskelynite/phosphate)</t>
-  </si>
-  <si>
     <t>25 nA</t>
   </si>
   <si>
     <t>20 nA</t>
-  </si>
-  <si>
-    <t>20 nA (X-ray maps/BSE); 20 nA silicates/sulfides/oxides; 8 nA phosphates; 4 nA carbonates</t>
-  </si>
-  <si>
-    <t>10 nA (carbonate/Mg,Na phosphate); 10 nA (oxides/olivine, 1 µm)</t>
   </si>
   <si>
     <t>EPMA Technique per Element</t>
@@ -1207,15 +1192,6 @@
   </si>
   <si>
     <t>parameter: DriftCorrection</t>
-  </si>
-  <si>
-    <t>Items marked 'Element Specific' in column F of this table become entries in the ada:analyteColumns Array.  a row in the analyte column array with name=BeamCurrentDefault</t>
-  </si>
-  <si>
-    <t>have to construct analyte template for properties associated with each analyte, defined in the analyteColumns Array, which is an array of schema:PropertyValueSpecification objects.The schema:valueName in the schema:PropertyValueSpecification becomes the (no namespace) keys in the elements in the default analytes array.  The base template only defines one analyteColumn: : ("schema:name": "Analysed Oxide-Element",
-        "schema:valueName": "element | oxide | isotope | isotopeRatio...etc",), and the default analytes array is simply an array like e.g. ("ada:defaultAnalytes": [
-      { "element": "Si"}, { "element": "Fe"},{ "element": "Mn"},... ]
-other columnss defined in the analyteColumn array are selected from the following 'Element specific' properties.</t>
   </si>
   <si>
     <t>analyteColumn : spectrometerNumber 
@@ -1414,14 +1390,6 @@
     <t>Match. analyte-level parameter with ada:enumeration of background correction methods (linear, exponential, mean of two points, etc.).</t>
   </si>
   <si>
-    <t>property:analyteTemplate
-  readOnly:true
-Dataset level parameter: reportedAnalyte
-  dataType: need 'analyte'  that is array of propertyValue? Or investigate DDI-CDI data point…These must be consistent with the method-level analyteTEmplate; they provide specific analyte-level reporting analtyteTemplate. In current model these would be the variableMeasured/Instance variables in the dataset metadata. The metod-level element-specific properties become additional properties on the measureVariable/PropertyValue.  
-For the element-specific properties, if a property is read only, it only need be specified in the tapp definition, not in the instance data, under the assumption that it always holds if this tapp is followed.
-User can add or delete an element when filling out the webform. Also, user should be allowed to copy and paste the filled content for different elements</t>
-  </si>
-  <si>
     <t>implementation notes</t>
   </si>
   <si>
@@ -1527,21 +1495,63 @@
   readOnly:True</t>
   </si>
   <si>
-    <t>property: : acceleratingVoltageDefault
+    <t>match. Same container as row 20 with ada:toolRole='reduction' for matrix-correction/data-reduction software.</t>
+  </si>
+  <si>
+    <t>MethodParameter (ada:fieldScope='method') , ada:dataType='number', schema:unitText='kV'</t>
+  </si>
+  <si>
+    <t>MethodParameter (ada:fieldScope='method') , ada:dataType='number', schema:unitText='um'.</t>
+  </si>
+  <si>
+    <t>parameter: BeamRasterDimenstion. 
+  dataType: schema:PropertyValue
+  readOnly: False</t>
+  </si>
+  <si>
+    <t>parameter:  BeamDamageMinimization. 
+  dataType:  text
+  readOnly: True</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> property: matrixCorrectionMethod
+  datatype: enum {PAP (Pouchou &amp; Pichoir Full) | XPP (Simplified PAP) | PhiRhoZ Bastin (EPQ-91) | Love-Scott I | Love-Scott II | Armstrong/Love-Scott | Heinrich/Duncumb-Reed | Conventional Philibert/Duncumb-Reed | Other | Unknown}
+   readOnly: true</t>
+  </si>
+  <si>
+    <t>$.ada:matrixCorrectionMethod</t>
+  </si>
+  <si>
+    <t>$MethodDefinition.ada:beamMode</t>
+  </si>
+  <si>
+    <t>$MethodDefinition.ada:acceleratingVoltageDefault</t>
+  </si>
+  <si>
+    <t>$MethodDefinition.ada:beamDiameterDefault</t>
+  </si>
+  <si>
+    <t>Method property (ada:fieldScope='method') with ada:enumeration of allowed values (focused|defocused|rastered) and ada:dataType='string'.</t>
+  </si>
+  <si>
+    <t>have to construct analyte template for properties associated with each analyte, defined in the analyteColumns Array, which is an array of schema:PropertyValueSpecification objects.The schema:valueName in the schema:PropertyValueSpecification becomes the (no namespace) keys in the elements in the default analytes array.  The base template only defines one analyteColumn: : ("schema:name": "Analysed Oxide-Element",
+        "schema:analyte",), and the default analytes array is simply an array like e.g. ("ada:defaultAnalytes": [
+      { "analyte": "Si"}, { "analyte": "Fe"},{ "analyte": "Mn"},... ]
+other columns defined in the analyteColumn array are selected from the following 'Analyte specific' properties.</t>
+  </si>
+  <si>
+    <t>Analyte specific</t>
+  </si>
+  <si>
+    <t>Items marked 'Analyte Specific' in column F of this table become entries in the ada:analyteColumns Array.  a row in the analyte column array with name=BeamCurrentDefault</t>
+  </si>
+  <si>
+    <t>property:  acceleratingVoltageDefault
   datatype: schema:PropertyValue
-  readonly True 
+  readonly: True 
 parameter: acceleratingVoltage
   dataType: schema:PropertyValue
-  parameter: readOnly: False</t>
-  </si>
-  <si>
-    <t>match. Same container as row 20 with ada:toolRole='reduction' for matrix-correction/data-reduction software.</t>
-  </si>
-  <si>
-    <t>MethodParameter (ada:fieldScope='method') , ada:dataType='number', schema:unitText='kV'</t>
-  </si>
-  <si>
-    <t>MethodParameter (ada:fieldScope='method') , ada:dataType='number', schema:unitText='um'.</t>
+  readOnly: False</t>
   </si>
   <si>
     <t>property: beamDiameterDefault
@@ -1549,37 +1559,56 @@
   dataType: schema:PropertyValue
 parameter: beamDiameter
   dataType: schema:PropertyValue
-  dataType: readOnly: False</t>
-  </si>
-  <si>
-    <t>parameter: BeamRasterDimenstion. 
-  dataType: schema:PropertyValue
   readOnly: False</t>
   </si>
   <si>
-    <t>parameter:  BeamDamageMinimization. 
-  dataType:  text
-  readOnly: True</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> property: matrixCorrectionMethod
-  datatype: enum {PAP (Pouchou &amp; Pichoir Full) | XPP (Simplified PAP) | PhiRhoZ Bastin (EPQ-91) | Love-Scott I | Love-Scott II | Armstrong/Love-Scott | Heinrich/Duncumb-Reed | Conventional Philibert/Duncumb-Reed | Other | Unknown}
-   readOnly: true</t>
-  </si>
-  <si>
-    <t>$.ada:matrixCorrectionMethod</t>
-  </si>
-  <si>
-    <t>$MethodDefinition.ada:beamMode</t>
-  </si>
-  <si>
-    <t>$MethodDefinition.ada:acceleratingVoltageDefault</t>
-  </si>
-  <si>
-    <t>$MethodDefinition.ada:beamDiameterDefault</t>
-  </si>
-  <si>
-    <t>Method property (ada:fieldScope='method') with ada:enumeration of allowed values (focused|defocused|rastered) and ada:dataType='string'.</t>
+    <t>property:analyteTemplate
+  readOnly: true
+Dataset level parameter: reportedAnalyte
+  dataType: need 'analyte'  that is array of propertyValue? Or investigate DDI-CDI data point…These must be consistent with the method-level analyteTEmplate; they provide specific analyte-level reporting analtyteTemplate. In current model these would be the variableMeasured/Instance variables in the dataset metadata. The metod-level element-specific properties become additional properties on the measureVariable/PropertyValue.  
+For the element-specific properties, if a property is read only, it only need be specified in the tapp definition, not in the instance data, under the assumption that it always holds if this tapp is followed.
+User can add or delete an element when filling out the webform. Also, user should be allowed to copy and paste the filled content for different elements</t>
+  </si>
+  <si>
+    <t>Asbestos microcline (Si Kα, Al Kα, K Kα);
+ Synthetic anorthite (Ca Kα); 
+Amelia albite (Na Kα); 
+Synthetic fayalite (Fe Kα); 
+Synthetic forsterite (Mg Kα); 
+Synthetic TiO2 (Ti Kα); 
+Synthetic Cr2O3 (Cr Kα); 
+Synthetic Mn-olivine (Mn Kα)</t>
+  </si>
+  <si>
+    <t>Anorthite (Si Kα, Al Kα, Ca Kα); 
+Albite (Na Kα); 
+Fayalite (Fe Kα); 
+Forsterite (Mg Kα); 
+Mn2SiO4 (Mn Kα); 
+TiO2 (Ti Kα); 
+Cr2O3 (Cr Kα); 
+Microcline (K Kα)</t>
+  </si>
+  <si>
+    <t>20 nA (X-ray maps/BSE); 
+20 nA silicates/sulfides/oxides;
+8 nA phosphates; 
+4 nA carbonates</t>
+  </si>
+  <si>
+    <t>20 nA (silicates/oxides); 
+10 nA (glass/maskelynite/phosphate)</t>
+  </si>
+  <si>
+    <t>10 nA (carbonate/Mg,Na phosphate); 
+10 nA (oxides/olivine, 1 µm)</t>
+  </si>
+  <si>
+    <t>Maskelynite, 
+melt inclusion glasses, 
+silica glass, 
+coesite aggregates, 
+mesostasis</t>
   </si>
 </sst>
 </file>
@@ -2892,16 +2921,19 @@
     <col min="2" max="2" width="33" style="58" customWidth="1"/>
     <col min="3" max="3" width="14.7109375" style="58" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.85546875" style="58" customWidth="1"/>
-    <col min="5" max="5" width="32" style="32" customWidth="1"/>
+    <col min="5" max="5" width="26.140625" style="32" customWidth="1"/>
     <col min="6" max="6" width="7.85546875" style="4" customWidth="1"/>
-    <col min="7" max="7" width="17.140625" style="4" customWidth="1"/>
-    <col min="8" max="8" width="38" style="167" hidden="1" customWidth="1"/>
-    <col min="9" max="12" width="38" style="58" hidden="1" customWidth="1"/>
-    <col min="13" max="17" width="30" style="58" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="8.42578125" style="168" customWidth="1"/>
+    <col min="7" max="7" width="28.28515625" style="4" customWidth="1"/>
+    <col min="8" max="8" width="28.28515625" style="167" customWidth="1"/>
+    <col min="9" max="9" width="28.28515625" style="58" customWidth="1"/>
+    <col min="10" max="10" width="36.85546875" style="58" customWidth="1"/>
+    <col min="11" max="14" width="28.28515625" style="58" customWidth="1"/>
+    <col min="15" max="15" width="33.42578125" style="58" customWidth="1"/>
+    <col min="16" max="17" width="28.28515625" style="58" customWidth="1"/>
+    <col min="18" max="18" width="28.28515625" style="168" customWidth="1"/>
     <col min="19" max="19" width="37.140625" style="4" customWidth="1"/>
     <col min="20" max="20" width="49.140625" style="4" customWidth="1"/>
-    <col min="21" max="21" width="49.5703125" style="4" customWidth="1"/>
+    <col min="21" max="21" width="56.5703125" style="4" customWidth="1"/>
     <col min="22" max="16384" width="12.7109375" style="4"/>
   </cols>
   <sheetData>
@@ -2922,7 +2954,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>424</v>
+        <v>416</v>
       </c>
       <c r="G1" s="2"/>
       <c r="H1" s="112" t="s">
@@ -2965,7 +2997,7 @@
         <v>17</v>
       </c>
       <c r="U1" s="3" t="s">
-        <v>414</v>
+        <v>406</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.2">
@@ -3046,10 +3078,10 @@
         <v>1</v>
       </c>
       <c r="S3" s="63" t="s">
-        <v>426</v>
+        <v>418</v>
       </c>
       <c r="T3" s="169" t="s">
-        <v>415</v>
+        <v>407</v>
       </c>
       <c r="U3" s="63"/>
     </row>
@@ -3106,13 +3138,13 @@
         <v>1</v>
       </c>
       <c r="S4" s="69" t="s">
-        <v>427</v>
+        <v>419</v>
       </c>
       <c r="T4" s="170" t="s">
-        <v>416</v>
+        <v>408</v>
       </c>
       <c r="U4" s="69" t="s">
-        <v>421</v>
+        <v>413</v>
       </c>
     </row>
     <row r="5" spans="1:21" s="70" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
@@ -3168,10 +3200,10 @@
         <v>1</v>
       </c>
       <c r="S5" s="69" t="s">
-        <v>428</v>
+        <v>420</v>
       </c>
       <c r="T5" s="170" t="s">
-        <v>417</v>
+        <v>409</v>
       </c>
       <c r="U5" s="69"/>
     </row>
@@ -3228,10 +3260,10 @@
         <v>1</v>
       </c>
       <c r="S6" s="69" t="s">
-        <v>429</v>
+        <v>421</v>
       </c>
       <c r="T6" s="170" t="s">
-        <v>418</v>
+        <v>410</v>
       </c>
       <c r="U6" s="69"/>
     </row>
@@ -3268,10 +3300,10 @@
         <v>0</v>
       </c>
       <c r="S7" s="69" t="s">
-        <v>430</v>
+        <v>422</v>
       </c>
       <c r="T7" s="170" t="s">
-        <v>439</v>
+        <v>431</v>
       </c>
       <c r="U7" s="69"/>
     </row>
@@ -3308,10 +3340,10 @@
         <v>0</v>
       </c>
       <c r="S8" s="69" t="s">
-        <v>431</v>
+        <v>423</v>
       </c>
       <c r="T8" s="170" t="s">
-        <v>419</v>
+        <v>411</v>
       </c>
       <c r="U8" s="69"/>
     </row>
@@ -3348,13 +3380,13 @@
         <v>0</v>
       </c>
       <c r="S9" s="69" t="s">
-        <v>432</v>
+        <v>424</v>
       </c>
       <c r="T9" s="170" t="s">
-        <v>420</v>
+        <v>412</v>
       </c>
       <c r="U9" s="69" t="s">
-        <v>422</v>
+        <v>414</v>
       </c>
     </row>
     <row r="10" spans="1:21" s="70" customFormat="1" ht="42.75" x14ac:dyDescent="0.2">
@@ -3390,10 +3422,10 @@
         <v>0</v>
       </c>
       <c r="S10" s="69" t="s">
-        <v>433</v>
+        <v>425</v>
       </c>
       <c r="T10" s="170" t="s">
-        <v>423</v>
+        <v>415</v>
       </c>
       <c r="U10" s="69"/>
     </row>
@@ -3445,7 +3477,7 @@
       <c r="T12" s="69"/>
       <c r="U12" s="69"/>
     </row>
-    <row r="13" spans="1:21" s="70" customFormat="1" ht="71.25" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:21" s="70" customFormat="1" ht="85.5" x14ac:dyDescent="0.2">
       <c r="A13" s="80" t="s">
         <v>74</v>
       </c>
@@ -3467,50 +3499,50 @@
         <v>78</v>
       </c>
       <c r="I13" s="81" t="s">
+        <v>462</v>
+      </c>
+      <c r="J13" s="81" t="s">
         <v>79</v>
       </c>
-      <c r="J13" s="81" t="s">
+      <c r="K13" s="81" t="s">
         <v>80</v>
       </c>
-      <c r="K13" s="81" t="s">
+      <c r="L13" s="81" t="s">
         <v>81</v>
       </c>
-      <c r="L13" s="81" t="s">
+      <c r="M13" s="81" t="s">
         <v>82</v>
       </c>
-      <c r="M13" s="81" t="s">
+      <c r="N13" s="81" t="s">
         <v>83</v>
       </c>
-      <c r="N13" s="81" t="s">
+      <c r="O13" s="81" t="s">
         <v>84</v>
       </c>
-      <c r="O13" s="81" t="s">
+      <c r="P13" s="81" t="s">
         <v>85</v>
       </c>
-      <c r="P13" s="81" t="s">
+      <c r="Q13" s="81" t="s">
         <v>86</v>
-      </c>
-      <c r="Q13" s="81" t="s">
-        <v>87</v>
       </c>
       <c r="R13" s="130">
         <f>COUNTA(H13:Q13)/10</f>
         <v>1</v>
       </c>
       <c r="S13" s="69" t="s">
-        <v>434</v>
+        <v>426</v>
       </c>
       <c r="T13" s="69" t="s">
-        <v>425</v>
+        <v>417</v>
       </c>
       <c r="U13" s="69"/>
     </row>
     <row r="14" spans="1:21" s="70" customFormat="1" ht="89.25" x14ac:dyDescent="0.2">
       <c r="A14" s="84" t="s">
+        <v>87</v>
+      </c>
+      <c r="B14" s="85" t="s">
         <v>88</v>
-      </c>
-      <c r="B14" s="85" t="s">
-        <v>89</v>
       </c>
       <c r="C14" s="86" t="s">
         <v>60</v>
@@ -3519,52 +3551,52 @@
         <v>22</v>
       </c>
       <c r="E14" s="87" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F14" s="69"/>
       <c r="G14" s="69"/>
       <c r="H14" s="131" t="s">
+        <v>90</v>
+      </c>
+      <c r="I14" s="85" t="s">
         <v>91</v>
       </c>
-      <c r="I14" s="85" t="s">
+      <c r="J14" s="85" t="s">
         <v>92</v>
       </c>
-      <c r="J14" s="85" t="s">
+      <c r="K14" s="85" t="s">
         <v>93</v>
       </c>
-      <c r="K14" s="85" t="s">
+      <c r="L14" s="85" t="s">
         <v>94</v>
       </c>
-      <c r="L14" s="85" t="s">
+      <c r="M14" s="85" t="s">
         <v>95</v>
       </c>
-      <c r="M14" s="85" t="s">
+      <c r="N14" s="85" t="s">
         <v>96</v>
       </c>
-      <c r="N14" s="85" t="s">
+      <c r="O14" s="85" t="s">
         <v>97</v>
       </c>
-      <c r="O14" s="85" t="s">
+      <c r="P14" s="85" t="s">
         <v>98</v>
       </c>
-      <c r="P14" s="85" t="s">
+      <c r="Q14" s="85" t="s">
         <v>99</v>
-      </c>
-      <c r="Q14" s="85" t="s">
-        <v>100</v>
       </c>
       <c r="R14" s="132">
         <f>COUNTA(H14:Q14)/10</f>
         <v>1</v>
       </c>
       <c r="S14" s="69" t="s">
-        <v>435</v>
+        <v>427</v>
       </c>
       <c r="T14" s="69" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="U14" s="69" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
     </row>
     <row r="15" spans="1:21" s="70" customFormat="1" ht="14.25" x14ac:dyDescent="0.2">
@@ -3592,7 +3624,7 @@
     </row>
     <row r="16" spans="1:21" s="70" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="178" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B16" s="176"/>
       <c r="C16" s="176"/>
@@ -3617,10 +3649,10 @@
     </row>
     <row r="17" spans="1:21" s="70" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A17" s="88" t="s">
+        <v>101</v>
+      </c>
+      <c r="B17" s="89" t="s">
         <v>102</v>
-      </c>
-      <c r="B17" s="89" t="s">
-        <v>103</v>
       </c>
       <c r="C17" s="90" t="s">
         <v>21</v>
@@ -3629,58 +3661,58 @@
         <v>31</v>
       </c>
       <c r="E17" s="91" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F17" s="69"/>
       <c r="G17" s="69"/>
       <c r="H17" s="133" t="s">
+        <v>104</v>
+      </c>
+      <c r="I17" s="89" t="s">
+        <v>104</v>
+      </c>
+      <c r="J17" s="89" t="s">
         <v>105</v>
       </c>
-      <c r="I17" s="89" t="s">
+      <c r="K17" s="89" t="s">
+        <v>104</v>
+      </c>
+      <c r="L17" s="89" t="s">
+        <v>106</v>
+      </c>
+      <c r="M17" s="89" t="s">
+        <v>104</v>
+      </c>
+      <c r="N17" s="89" t="s">
+        <v>104</v>
+      </c>
+      <c r="O17" s="89" t="s">
         <v>105</v>
       </c>
-      <c r="J17" s="89" t="s">
-        <v>106</v>
-      </c>
-      <c r="K17" s="89" t="s">
-        <v>105</v>
-      </c>
-      <c r="L17" s="89" t="s">
+      <c r="P17" s="89" t="s">
         <v>107</v>
       </c>
-      <c r="M17" s="89" t="s">
-        <v>105</v>
-      </c>
-      <c r="N17" s="89" t="s">
-        <v>105</v>
-      </c>
-      <c r="O17" s="89" t="s">
-        <v>106</v>
-      </c>
-      <c r="P17" s="89" t="s">
-        <v>108</v>
-      </c>
       <c r="Q17" s="89" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="R17" s="134">
         <f t="shared" ref="R17:R23" si="1">COUNTA(H17:Q17)/10</f>
         <v>1</v>
       </c>
       <c r="S17" s="69" t="s">
-        <v>436</v>
+        <v>428</v>
       </c>
       <c r="T17" s="170" t="s">
-        <v>437</v>
+        <v>429</v>
       </c>
       <c r="U17" s="69"/>
     </row>
     <row r="18" spans="1:21" s="70" customFormat="1" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A18" s="88" t="s">
+        <v>108</v>
+      </c>
+      <c r="B18" s="89" t="s">
         <v>109</v>
-      </c>
-      <c r="B18" s="89" t="s">
-        <v>110</v>
       </c>
       <c r="C18" s="90" t="s">
         <v>21</v>
@@ -3689,58 +3721,58 @@
         <v>31</v>
       </c>
       <c r="E18" s="91" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F18" s="69"/>
       <c r="G18" s="69"/>
       <c r="H18" s="133" t="s">
+        <v>111</v>
+      </c>
+      <c r="I18" s="89" t="s">
         <v>112</v>
       </c>
-      <c r="I18" s="89" t="s">
+      <c r="J18" s="89" t="s">
         <v>113</v>
       </c>
-      <c r="J18" s="89" t="s">
+      <c r="K18" s="89" t="s">
+        <v>111</v>
+      </c>
+      <c r="L18" s="89" t="s">
         <v>114</v>
       </c>
-      <c r="K18" s="89" t="s">
-        <v>112</v>
-      </c>
-      <c r="L18" s="89" t="s">
+      <c r="M18" s="89" t="s">
+        <v>111</v>
+      </c>
+      <c r="N18" s="89" t="s">
         <v>115</v>
       </c>
-      <c r="M18" s="89" t="s">
-        <v>112</v>
-      </c>
-      <c r="N18" s="89" t="s">
+      <c r="O18" s="89" t="s">
         <v>116</v>
       </c>
-      <c r="O18" s="89" t="s">
+      <c r="P18" s="89" t="s">
         <v>117</v>
       </c>
-      <c r="P18" s="89" t="s">
+      <c r="Q18" s="89" t="s">
         <v>118</v>
-      </c>
-      <c r="Q18" s="89" t="s">
-        <v>119</v>
       </c>
       <c r="R18" s="134">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="S18" s="69" t="s">
-        <v>442</v>
+        <v>434</v>
       </c>
       <c r="T18" s="170" t="s">
-        <v>438</v>
+        <v>430</v>
       </c>
       <c r="U18" s="69"/>
     </row>
     <row r="19" spans="1:21" s="70" customFormat="1" ht="51" x14ac:dyDescent="0.2">
       <c r="A19" s="88" t="s">
+        <v>119</v>
+      </c>
+      <c r="B19" s="89" t="s">
         <v>120</v>
-      </c>
-      <c r="B19" s="89" t="s">
-        <v>121</v>
       </c>
       <c r="C19" s="90" t="s">
         <v>21</v>
@@ -3749,7 +3781,7 @@
         <v>31</v>
       </c>
       <c r="E19" s="91" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F19" s="69"/>
       <c r="G19" s="69"/>
@@ -3760,11 +3792,11 @@
       <c r="L19" s="89"/>
       <c r="M19" s="89"/>
       <c r="N19" s="89" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="O19" s="89"/>
       <c r="P19" s="89" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="Q19" s="89"/>
       <c r="R19" s="134">
@@ -3772,19 +3804,19 @@
         <v>0.2</v>
       </c>
       <c r="S19" s="69" t="s">
-        <v>443</v>
+        <v>435</v>
       </c>
       <c r="T19" s="69" t="s">
-        <v>440</v>
+        <v>432</v>
       </c>
       <c r="U19" s="69"/>
     </row>
     <row r="20" spans="1:21" s="70" customFormat="1" ht="51" x14ac:dyDescent="0.2">
       <c r="A20" s="88" t="s">
+        <v>123</v>
+      </c>
+      <c r="B20" s="89" t="s">
         <v>124</v>
-      </c>
-      <c r="B20" s="89" t="s">
-        <v>125</v>
       </c>
       <c r="C20" s="90" t="s">
         <v>21</v>
@@ -3793,25 +3825,25 @@
         <v>22</v>
       </c>
       <c r="E20" s="91" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F20" s="69"/>
       <c r="G20" s="69"/>
       <c r="H20" s="133" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I20" s="89"/>
       <c r="J20" s="89"/>
       <c r="K20" s="89" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="L20" s="89"/>
       <c r="M20" s="89" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="N20" s="89"/>
       <c r="O20" s="89" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="P20" s="89"/>
       <c r="Q20" s="89"/>
@@ -3820,75 +3852,75 @@
         <v>0.4</v>
       </c>
       <c r="S20" s="69" t="s">
-        <v>444</v>
+        <v>436</v>
       </c>
       <c r="T20" s="170" t="s">
-        <v>441</v>
+        <v>433</v>
       </c>
       <c r="U20" s="69" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
     </row>
     <row r="21" spans="1:21" s="70" customFormat="1" ht="57" x14ac:dyDescent="0.2">
       <c r="A21" s="88" t="s">
+        <v>128</v>
+      </c>
+      <c r="B21" s="89" t="s">
         <v>129</v>
-      </c>
-      <c r="B21" s="89" t="s">
-        <v>130</v>
       </c>
       <c r="C21" s="90" t="s">
         <v>21</v>
       </c>
       <c r="D21" s="89" t="s">
+        <v>130</v>
+      </c>
+      <c r="E21" s="91" t="s">
         <v>131</v>
-      </c>
-      <c r="E21" s="91" t="s">
-        <v>132</v>
       </c>
       <c r="F21" s="69"/>
       <c r="G21" s="69"/>
       <c r="H21" s="133" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I21" s="89"/>
       <c r="J21" s="89"/>
       <c r="K21" s="89" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="L21" s="89"/>
       <c r="M21" s="89" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="N21" s="89"/>
       <c r="O21" s="89" t="s">
+        <v>134</v>
+      </c>
+      <c r="P21" s="89" t="s">
         <v>135</v>
       </c>
-      <c r="P21" s="89" t="s">
-        <v>136</v>
-      </c>
       <c r="Q21" s="89" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="R21" s="134">
         <f t="shared" si="1"/>
         <v>0.6</v>
       </c>
       <c r="S21" s="69" t="s">
-        <v>444</v>
+        <v>436</v>
       </c>
       <c r="T21" s="170" t="s">
-        <v>449</v>
+        <v>440</v>
       </c>
       <c r="U21" s="69" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
     </row>
     <row r="22" spans="1:21" s="70" customFormat="1" ht="57" x14ac:dyDescent="0.2">
       <c r="A22" s="92" t="s">
+        <v>136</v>
+      </c>
+      <c r="B22" s="93" t="s">
         <v>137</v>
-      </c>
-      <c r="B22" s="93" t="s">
-        <v>138</v>
       </c>
       <c r="C22" s="94" t="s">
         <v>60</v>
@@ -3897,7 +3929,7 @@
         <v>22</v>
       </c>
       <c r="E22" s="95" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F22" s="69"/>
       <c r="G22" s="69"/>
@@ -3907,7 +3939,7 @@
       <c r="K22" s="93"/>
       <c r="L22" s="93"/>
       <c r="M22" s="93" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="N22" s="93"/>
       <c r="O22" s="93"/>
@@ -3918,21 +3950,21 @@
         <v>0.1</v>
       </c>
       <c r="S22" s="69" t="s">
-        <v>443</v>
+        <v>435</v>
       </c>
       <c r="T22" s="69" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="U22" s="69" t="s">
-        <v>446</v>
+        <v>438</v>
       </c>
     </row>
     <row r="23" spans="1:21" s="70" customFormat="1" ht="51" x14ac:dyDescent="0.2">
       <c r="A23" s="92" t="s">
+        <v>141</v>
+      </c>
+      <c r="B23" s="93" t="s">
         <v>142</v>
-      </c>
-      <c r="B23" s="93" t="s">
-        <v>143</v>
       </c>
       <c r="C23" s="94" t="s">
         <v>60</v>
@@ -3941,7 +3973,7 @@
         <v>22</v>
       </c>
       <c r="E23" s="95" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F23" s="69"/>
       <c r="G23" s="69"/>
@@ -3951,7 +3983,7 @@
       <c r="K23" s="93"/>
       <c r="L23" s="93"/>
       <c r="M23" s="93" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="N23" s="93"/>
       <c r="O23" s="93"/>
@@ -3962,13 +3994,13 @@
         <v>0.1</v>
       </c>
       <c r="S23" s="69" t="s">
-        <v>443</v>
+        <v>435</v>
       </c>
       <c r="T23" s="69" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="U23" s="69" t="s">
-        <v>445</v>
+        <v>437</v>
       </c>
     </row>
     <row r="24" spans="1:21" s="70" customFormat="1" ht="14.25" x14ac:dyDescent="0.2">
@@ -3996,7 +4028,7 @@
     </row>
     <row r="25" spans="1:21" s="70" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A25" s="179" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B25" s="176"/>
       <c r="C25" s="176"/>
@@ -4021,10 +4053,10 @@
     </row>
     <row r="26" spans="1:21" s="70" customFormat="1" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A26" s="96" t="s">
+        <v>147</v>
+      </c>
+      <c r="B26" s="97" t="s">
         <v>148</v>
-      </c>
-      <c r="B26" s="97" t="s">
-        <v>149</v>
       </c>
       <c r="C26" s="98" t="s">
         <v>21</v>
@@ -4033,191 +4065,191 @@
         <v>31</v>
       </c>
       <c r="E26" s="99" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F26" s="69"/>
       <c r="G26" s="69"/>
       <c r="H26" s="137" t="s">
+        <v>150</v>
+      </c>
+      <c r="I26" s="97" t="s">
+        <v>150</v>
+      </c>
+      <c r="J26" s="97" t="s">
         <v>151</v>
       </c>
-      <c r="I26" s="97" t="s">
-        <v>151</v>
-      </c>
-      <c r="J26" s="97" t="s">
+      <c r="K26" s="97" t="s">
+        <v>150</v>
+      </c>
+      <c r="L26" s="97" t="s">
+        <v>150</v>
+      </c>
+      <c r="M26" s="97" t="s">
+        <v>150</v>
+      </c>
+      <c r="N26" s="97" t="s">
         <v>152</v>
       </c>
-      <c r="K26" s="97" t="s">
-        <v>151</v>
-      </c>
-      <c r="L26" s="97" t="s">
-        <v>151</v>
-      </c>
-      <c r="M26" s="97" t="s">
-        <v>151</v>
-      </c>
-      <c r="N26" s="97" t="s">
+      <c r="O26" s="97" t="s">
         <v>153</v>
       </c>
-      <c r="O26" s="97" t="s">
+      <c r="P26" s="97" t="s">
         <v>154</v>
       </c>
-      <c r="P26" s="97" t="s">
+      <c r="Q26" s="97" t="s">
         <v>155</v>
-      </c>
-      <c r="Q26" s="97" t="s">
-        <v>156</v>
       </c>
       <c r="R26" s="138">
         <f t="shared" ref="R26:R43" si="2">COUNTA(H26:Q26)/10</f>
         <v>1</v>
       </c>
       <c r="S26" s="69" t="s">
-        <v>457</v>
+        <v>447</v>
       </c>
       <c r="T26" s="170" t="s">
-        <v>460</v>
+        <v>450</v>
       </c>
       <c r="U26" s="171" t="s">
-        <v>447</v>
+        <v>439</v>
       </c>
     </row>
     <row r="27" spans="1:21" s="70" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A27" s="96" t="s">
+        <v>157</v>
+      </c>
+      <c r="B27" s="97" t="s">
         <v>158</v>
-      </c>
-      <c r="B27" s="97" t="s">
-        <v>159</v>
       </c>
       <c r="C27" s="100" t="s">
         <v>21</v>
       </c>
       <c r="D27" s="97" t="s">
+        <v>159</v>
+      </c>
+      <c r="E27" s="99" t="s">
         <v>160</v>
-      </c>
-      <c r="E27" s="99" t="s">
-        <v>161</v>
       </c>
       <c r="F27" s="69"/>
       <c r="G27" s="69"/>
       <c r="H27" s="137" t="s">
+        <v>161</v>
+      </c>
+      <c r="I27" s="97" t="s">
+        <v>161</v>
+      </c>
+      <c r="J27" s="97" t="s">
+        <v>161</v>
+      </c>
+      <c r="K27" s="97" t="s">
+        <v>161</v>
+      </c>
+      <c r="L27" s="97" t="s">
         <v>162</v>
       </c>
-      <c r="I27" s="97" t="s">
-        <v>162</v>
-      </c>
-      <c r="J27" s="97" t="s">
-        <v>162</v>
-      </c>
-      <c r="K27" s="97" t="s">
-        <v>162</v>
-      </c>
-      <c r="L27" s="97" t="s">
-        <v>163</v>
-      </c>
       <c r="M27" s="97" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="N27" s="97" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="O27" s="97" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="P27" s="97" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="Q27" s="97" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="R27" s="138">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="S27" s="101" t="s">
-        <v>458</v>
+        <v>448</v>
       </c>
       <c r="T27" s="170" t="s">
-        <v>450</v>
+        <v>441</v>
       </c>
       <c r="U27" s="171" t="s">
-        <v>448</v>
+        <v>454</v>
       </c>
     </row>
     <row r="28" spans="1:21" s="70" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
       <c r="A28" s="96" t="s">
+        <v>164</v>
+      </c>
+      <c r="B28" s="97" t="s">
         <v>165</v>
-      </c>
-      <c r="B28" s="97" t="s">
-        <v>166</v>
       </c>
       <c r="C28" s="100" t="s">
         <v>21</v>
       </c>
       <c r="D28" s="97" t="s">
+        <v>166</v>
+      </c>
+      <c r="E28" s="99" t="s">
         <v>167</v>
-      </c>
-      <c r="E28" s="99" t="s">
-        <v>168</v>
       </c>
       <c r="F28" s="69"/>
       <c r="G28" s="69"/>
       <c r="H28" s="137" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="I28" s="97"/>
       <c r="J28" s="97" t="s">
+        <v>169</v>
+      </c>
+      <c r="K28" s="97" t="s">
+        <v>168</v>
+      </c>
+      <c r="L28" s="97" t="s">
         <v>170</v>
       </c>
-      <c r="K28" s="97" t="s">
-        <v>169</v>
-      </c>
-      <c r="L28" s="97" t="s">
+      <c r="M28" s="97" t="s">
+        <v>168</v>
+      </c>
+      <c r="N28" s="97" t="s">
         <v>171</v>
       </c>
-      <c r="M28" s="97" t="s">
-        <v>169</v>
-      </c>
-      <c r="N28" s="97" t="s">
+      <c r="O28" s="97" t="s">
         <v>172</v>
       </c>
-      <c r="O28" s="97" t="s">
+      <c r="P28" s="97" t="s">
         <v>173</v>
       </c>
-      <c r="P28" s="97" t="s">
+      <c r="Q28" s="97" t="s">
         <v>174</v>
-      </c>
-      <c r="Q28" s="97" t="s">
-        <v>175</v>
       </c>
       <c r="R28" s="138">
         <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
       <c r="S28" s="101" t="s">
-        <v>459</v>
+        <v>449</v>
       </c>
       <c r="T28" s="170" t="s">
-        <v>451</v>
+        <v>442</v>
       </c>
       <c r="U28" s="171" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
     </row>
     <row r="29" spans="1:21" s="70" customFormat="1" ht="51" x14ac:dyDescent="0.2">
       <c r="A29" s="102" t="s">
+        <v>175</v>
+      </c>
+      <c r="B29" s="103" t="s">
         <v>176</v>
-      </c>
-      <c r="B29" s="103" t="s">
-        <v>177</v>
       </c>
       <c r="C29" s="104" t="s">
         <v>60</v>
       </c>
       <c r="D29" s="103" t="s">
+        <v>177</v>
+      </c>
+      <c r="E29" s="105" t="s">
         <v>178</v>
-      </c>
-      <c r="E29" s="105" t="s">
-        <v>179</v>
       </c>
       <c r="F29" s="69"/>
       <c r="G29" s="69"/>
@@ -4236,21 +4268,21 @@
         <v>0</v>
       </c>
       <c r="S29" s="69" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="T29" s="69" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="U29" s="69" t="s">
-        <v>453</v>
+        <v>443</v>
       </c>
     </row>
     <row r="30" spans="1:21" s="70" customFormat="1" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A30" s="102" t="s">
+        <v>180</v>
+      </c>
+      <c r="B30" s="103" t="s">
         <v>181</v>
-      </c>
-      <c r="B30" s="103" t="s">
-        <v>182</v>
       </c>
       <c r="C30" s="104" t="s">
         <v>60</v>
@@ -4259,7 +4291,7 @@
         <v>22</v>
       </c>
       <c r="E30" s="105" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F30" s="69"/>
       <c r="G30" s="69"/>
@@ -4269,10 +4301,10 @@
       <c r="K30" s="103"/>
       <c r="L30" s="103"/>
       <c r="M30" s="103" t="s">
+        <v>183</v>
+      </c>
+      <c r="N30" s="103" t="s">
         <v>184</v>
-      </c>
-      <c r="N30" s="103" t="s">
-        <v>185</v>
       </c>
       <c r="O30" s="103"/>
       <c r="P30" s="103"/>
@@ -4282,21 +4314,21 @@
         <v>0.2</v>
       </c>
       <c r="S30" s="69" t="s">
+        <v>185</v>
+      </c>
+      <c r="T30" s="69" t="s">
         <v>186</v>
       </c>
-      <c r="T30" s="69" t="s">
-        <v>187</v>
-      </c>
       <c r="U30" s="69" t="s">
-        <v>454</v>
+        <v>444</v>
       </c>
     </row>
     <row r="31" spans="1:21" s="111" customFormat="1" ht="72" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A31" s="106" t="s">
+        <v>187</v>
+      </c>
+      <c r="B31" s="107" t="s">
         <v>188</v>
-      </c>
-      <c r="B31" s="107" t="s">
-        <v>189</v>
       </c>
       <c r="C31" s="108" t="s">
         <v>60</v>
@@ -4305,7 +4337,7 @@
         <v>22</v>
       </c>
       <c r="E31" s="109" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F31" s="110"/>
       <c r="G31" s="110"/>
@@ -4324,21 +4356,21 @@
         <v>0</v>
       </c>
       <c r="S31" s="110" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="T31" s="110" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="U31" s="110" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
     </row>
     <row r="32" spans="1:21" ht="234" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="B32" s="36" t="s">
         <v>192</v>
-      </c>
-      <c r="B32" s="36" t="s">
-        <v>193</v>
       </c>
       <c r="C32" s="37" t="s">
         <v>21</v>
@@ -4347,11 +4379,11 @@
         <v>31</v>
       </c>
       <c r="E32" s="21" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F32" s="3"/>
       <c r="G32" s="3" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="H32" s="143"/>
       <c r="I32" s="36"/>
@@ -4368,85 +4400,85 @@
         <v>0</v>
       </c>
       <c r="S32" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="T32" s="3" t="s">
-        <v>369</v>
+        <v>451</v>
       </c>
       <c r="U32" s="3" t="s">
-        <v>413</v>
+        <v>456</v>
       </c>
     </row>
     <row r="33" spans="1:21" ht="77.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A33" s="12" t="s">
+        <v>196</v>
+      </c>
+      <c r="B33" s="36" t="s">
         <v>197</v>
-      </c>
-      <c r="B33" s="36" t="s">
-        <v>198</v>
       </c>
       <c r="C33" s="38" t="s">
         <v>21</v>
       </c>
       <c r="D33" s="36" t="s">
+        <v>198</v>
+      </c>
+      <c r="E33" s="21" t="s">
         <v>199</v>
       </c>
-      <c r="E33" s="21" t="s">
-        <v>200</v>
-      </c>
       <c r="F33" s="3" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G33" s="3"/>
       <c r="H33" s="143" t="s">
+        <v>200</v>
+      </c>
+      <c r="I33" s="36" t="s">
+        <v>201</v>
+      </c>
+      <c r="J33" s="36" t="s">
+        <v>460</v>
+      </c>
+      <c r="K33" s="36" t="s">
+        <v>200</v>
+      </c>
+      <c r="L33" s="36" t="s">
+        <v>162</v>
+      </c>
+      <c r="M33" s="36" t="s">
         <v>202</v>
       </c>
-      <c r="I33" s="36" t="s">
+      <c r="N33" s="36" t="s">
         <v>203</v>
       </c>
-      <c r="J33" s="36" t="s">
-        <v>204</v>
-      </c>
-      <c r="K33" s="36" t="s">
-        <v>202</v>
-      </c>
-      <c r="L33" s="36" t="s">
-        <v>163</v>
-      </c>
-      <c r="M33" s="36" t="s">
-        <v>205</v>
-      </c>
-      <c r="N33" s="36" t="s">
-        <v>206</v>
-      </c>
       <c r="O33" s="36" t="s">
-        <v>207</v>
+        <v>459</v>
       </c>
       <c r="P33" s="36" t="s">
-        <v>208</v>
+        <v>461</v>
       </c>
       <c r="Q33" s="36" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="R33" s="144">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="S33" s="11" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="T33" s="3" t="s">
-        <v>368</v>
+        <v>453</v>
       </c>
       <c r="U33" s="3" t="s">
-        <v>372</v>
+        <v>365</v>
       </c>
     </row>
     <row r="34" spans="1:21" ht="39" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="B34" s="36" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="C34" s="38" t="s">
         <v>21</v>
@@ -4455,74 +4487,74 @@
         <v>31</v>
       </c>
       <c r="E34" s="21" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G34" s="3"/>
       <c r="H34" s="143" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="I34" s="36" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="J34" s="36" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="K34" s="36" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="L34" s="36" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="M34" s="36" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="N34" s="36" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="O34" s="36" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="P34" s="36" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="Q34" s="36" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="R34" s="144">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="S34" s="11" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="T34" s="3" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="U34" s="3" t="s">
-        <v>373</v>
+        <v>366</v>
       </c>
     </row>
     <row r="35" spans="1:21" ht="39" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A35" s="13" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="B35" s="39" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="C35" s="40" t="s">
         <v>60</v>
       </c>
       <c r="D35" s="39" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="E35" s="22" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G35" s="3"/>
       <c r="H35" s="145"/>
@@ -4540,33 +4572,33 @@
         <v>0</v>
       </c>
       <c r="S35" s="3" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="T35" s="3" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="U35" s="3" t="s">
-        <v>370</v>
+        <v>363</v>
       </c>
     </row>
     <row r="36" spans="1:21" ht="39" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A36" s="13" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="B36" s="39" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C36" s="40" t="s">
         <v>60</v>
       </c>
       <c r="D36" s="39" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="E36" s="22" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G36" s="3"/>
       <c r="H36" s="145"/>
@@ -4584,21 +4616,21 @@
         <v>0</v>
       </c>
       <c r="S36" s="3" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="T36" s="3" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="U36" s="3" t="s">
-        <v>371</v>
+        <v>364</v>
       </c>
     </row>
     <row r="37" spans="1:21" ht="72" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="B37" s="36" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="C37" s="37" t="s">
         <v>21</v>
@@ -4607,10 +4639,10 @@
         <v>31</v>
       </c>
       <c r="E37" s="21" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G37" s="3"/>
       <c r="H37" s="143"/>
@@ -4619,7 +4651,7 @@
       <c r="K37" s="36"/>
       <c r="L37" s="36"/>
       <c r="M37" s="36" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="N37" s="36"/>
       <c r="O37" s="36"/>
@@ -4630,21 +4662,21 @@
         <v>0.1</v>
       </c>
       <c r="S37" s="3" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="T37" s="3" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="U37" s="3" t="s">
-        <v>374</v>
+        <v>367</v>
       </c>
     </row>
     <row r="38" spans="1:21" ht="64.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A38" s="13" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="B38" s="39" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="C38" s="40" t="s">
         <v>60</v>
@@ -4653,10 +4685,10 @@
         <v>31</v>
       </c>
       <c r="E38" s="22" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G38" s="3"/>
       <c r="H38" s="145"/>
@@ -4674,21 +4706,21 @@
         <v>0</v>
       </c>
       <c r="S38" s="3" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="T38" s="3" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="U38" s="3" t="s">
-        <v>375</v>
+        <v>368</v>
       </c>
     </row>
     <row r="39" spans="1:21" ht="39" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A39" s="13" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="B39" s="39" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="C39" s="40" t="s">
         <v>60</v>
@@ -4697,10 +4729,10 @@
         <v>31</v>
       </c>
       <c r="E39" s="22" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G39" s="3"/>
       <c r="H39" s="145"/>
@@ -4718,21 +4750,21 @@
         <v>0</v>
       </c>
       <c r="S39" s="3" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="T39" s="3" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="U39" s="3" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="40" spans="1:21" ht="100.5" thickBot="1" x14ac:dyDescent="0.25">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="40" spans="1:21" ht="129" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A40" s="12" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="B40" s="36" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="C40" s="38" t="s">
         <v>21</v>
@@ -4741,19 +4773,19 @@
         <v>31</v>
       </c>
       <c r="E40" s="21" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G40" s="3"/>
       <c r="H40" s="143" t="s">
-        <v>239</v>
+        <v>458</v>
       </c>
       <c r="I40" s="36"/>
       <c r="J40" s="36"/>
       <c r="K40" s="36" t="s">
-        <v>240</v>
+        <v>457</v>
       </c>
       <c r="L40" s="36"/>
       <c r="M40" s="36"/>
@@ -4766,52 +4798,52 @@
         <v>0.2</v>
       </c>
       <c r="S40" s="11" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="T40" s="3" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="U40" s="3" t="s">
-        <v>377</v>
+        <v>370</v>
       </c>
     </row>
     <row r="41" spans="1:21" ht="57.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A41" s="12" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="B41" s="36" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="C41" s="38" t="s">
         <v>21</v>
       </c>
       <c r="D41" s="36" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="E41" s="21" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G41" s="3"/>
       <c r="H41" s="143" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I41" s="36"/>
       <c r="J41" s="36"/>
       <c r="K41" s="36" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L41" s="36" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="M41" s="36"/>
       <c r="N41" s="36" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="O41" s="36" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="P41" s="36"/>
       <c r="Q41" s="36"/>
@@ -4820,50 +4852,50 @@
         <v>0.5</v>
       </c>
       <c r="S41" s="11" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="T41" s="3" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="U41" s="3" t="s">
-        <v>378</v>
+        <v>371</v>
       </c>
     </row>
     <row r="42" spans="1:21" ht="57.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A42" s="12" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="B42" s="36" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="C42" s="38" t="s">
         <v>21</v>
       </c>
       <c r="D42" s="36" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="E42" s="21" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G42" s="3"/>
       <c r="H42" s="143" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="I42" s="36"/>
       <c r="J42" s="36"/>
       <c r="K42" s="36" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="L42" s="36"/>
       <c r="M42" s="36"/>
       <c r="N42" s="36" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="O42" s="36" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="P42" s="36"/>
       <c r="Q42" s="36"/>
@@ -4872,33 +4904,33 @@
         <v>0.4</v>
       </c>
       <c r="S42" s="11" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="T42" s="3" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="U42" s="3" t="s">
-        <v>379</v>
+        <v>372</v>
       </c>
     </row>
     <row r="43" spans="1:21" ht="72" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A43" s="13" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="B43" s="39" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="C43" s="40" t="s">
         <v>60</v>
       </c>
       <c r="D43" s="39" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="E43" s="22" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G43" s="3"/>
       <c r="H43" s="145"/>
@@ -4916,13 +4948,13 @@
         <v>0</v>
       </c>
       <c r="S43" s="3" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="T43" s="3" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="U43" s="3" t="s">
-        <v>380</v>
+        <v>373</v>
       </c>
     </row>
     <row r="44" spans="1:21" ht="14.25" x14ac:dyDescent="0.2">
@@ -4950,7 +4982,7 @@
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A45" s="180" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="B45" s="173"/>
       <c r="C45" s="173"/>
@@ -4975,10 +5007,10 @@
     </row>
     <row r="46" spans="1:21" ht="114" x14ac:dyDescent="0.2">
       <c r="A46" s="6" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="B46" s="41" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="C46" s="35" t="s">
         <v>21</v>
@@ -4987,54 +5019,54 @@
         <v>31</v>
       </c>
       <c r="E46" s="23" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="F46" s="3"/>
       <c r="G46" s="3"/>
       <c r="H46" s="147" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="I46" s="41" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="J46" s="41"/>
       <c r="K46" s="41" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="L46" s="41"/>
       <c r="M46" s="41" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="N46" s="41"/>
       <c r="O46" s="41" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="P46" s="41" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="Q46" s="41" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="R46" s="148">
         <f t="shared" ref="R46:R56" si="3">COUNTA(H46:Q46)/10</f>
         <v>0.7</v>
       </c>
       <c r="S46" s="11" t="s">
-        <v>456</v>
+        <v>446</v>
       </c>
       <c r="T46" s="3" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="U46" s="3" t="s">
-        <v>455</v>
+        <v>445</v>
       </c>
     </row>
     <row r="47" spans="1:21" ht="51" x14ac:dyDescent="0.2">
       <c r="A47" s="6" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="B47" s="41" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="C47" s="42" t="s">
         <v>21</v>
@@ -5043,7 +5075,7 @@
         <v>31</v>
       </c>
       <c r="E47" s="23" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="F47" s="3"/>
       <c r="G47" s="3"/>
@@ -5062,30 +5094,30 @@
         <v>0</v>
       </c>
       <c r="S47" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="T47" s="3" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="U47" s="3" t="s">
-        <v>381</v>
+        <v>374</v>
       </c>
     </row>
     <row r="48" spans="1:21" ht="57" x14ac:dyDescent="0.2">
       <c r="A48" s="7" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="B48" s="43" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="C48" s="44" t="s">
         <v>60</v>
       </c>
       <c r="D48" s="43" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="E48" s="24" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="F48" s="3"/>
       <c r="G48" s="3"/>
@@ -5095,10 +5127,10 @@
       <c r="K48" s="43"/>
       <c r="L48" s="43"/>
       <c r="M48" s="43" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="N48" s="43" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="O48" s="43"/>
       <c r="P48" s="43"/>
@@ -5108,21 +5140,21 @@
         <v>0.2</v>
       </c>
       <c r="S48" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="T48" s="3" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="U48" s="3" t="s">
-        <v>382</v>
+        <v>375</v>
       </c>
     </row>
     <row r="49" spans="1:21" ht="99.75" x14ac:dyDescent="0.2">
       <c r="A49" s="6" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="B49" s="41" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="C49" s="42" t="s">
         <v>21</v>
@@ -5131,7 +5163,7 @@
         <v>31</v>
       </c>
       <c r="E49" s="23" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="F49" s="3"/>
       <c r="G49" s="3"/>
@@ -5150,21 +5182,21 @@
         <v>0</v>
       </c>
       <c r="S49" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="T49" s="3" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="U49" s="3" t="s">
-        <v>383</v>
+        <v>376</v>
       </c>
     </row>
     <row r="50" spans="1:21" ht="64.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A50" s="7" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="B50" s="43" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="C50" s="44" t="s">
         <v>60</v>
@@ -5173,7 +5205,7 @@
         <v>31</v>
       </c>
       <c r="E50" s="24" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="F50" s="3"/>
       <c r="G50" s="3"/>
@@ -5192,21 +5224,21 @@
         <v>0</v>
       </c>
       <c r="S50" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="T50" s="3" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="U50" s="3" t="s">
-        <v>384</v>
+        <v>377</v>
       </c>
     </row>
     <row r="51" spans="1:21" ht="43.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="B51" s="45" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="C51" s="46" t="s">
         <v>60</v>
@@ -5215,10 +5247,10 @@
         <v>22</v>
       </c>
       <c r="E51" s="25" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G51" s="3"/>
       <c r="H51" s="151"/>
@@ -5236,21 +5268,21 @@
         <v>0</v>
       </c>
       <c r="S51" s="3" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="T51" s="3" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="U51" s="3" t="s">
-        <v>385</v>
+        <v>378</v>
       </c>
     </row>
     <row r="52" spans="1:21" ht="43.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="B52" s="45" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="C52" s="46" t="s">
         <v>60</v>
@@ -5259,10 +5291,10 @@
         <v>22</v>
       </c>
       <c r="E52" s="25" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G52" s="3"/>
       <c r="H52" s="151"/>
@@ -5280,21 +5312,21 @@
         <v>0</v>
       </c>
       <c r="S52" s="3" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="T52" s="3" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="U52" s="3" t="s">
-        <v>386</v>
+        <v>379</v>
       </c>
     </row>
     <row r="53" spans="1:21" ht="39" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A53" s="15" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="B53" s="47" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="C53" s="48" t="s">
         <v>60</v>
@@ -5303,10 +5335,10 @@
         <v>22</v>
       </c>
       <c r="E53" s="26" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G53" s="3"/>
       <c r="H53" s="153"/>
@@ -5324,21 +5356,21 @@
         <v>0</v>
       </c>
       <c r="S53" s="3" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="T53" s="3" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="U53" s="3" t="s">
-        <v>387</v>
+        <v>380</v>
       </c>
     </row>
     <row r="54" spans="1:21" ht="114.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="16" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="B54" s="49" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="C54" s="38" t="s">
         <v>21</v>
@@ -5347,10 +5379,10 @@
         <v>31</v>
       </c>
       <c r="E54" s="27" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G54" s="3"/>
       <c r="H54" s="155"/>
@@ -5359,7 +5391,7 @@
       <c r="K54" s="49"/>
       <c r="L54" s="49"/>
       <c r="M54" s="49" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="N54" s="49"/>
       <c r="O54" s="49"/>
@@ -5370,21 +5402,21 @@
         <v>0.1</v>
       </c>
       <c r="S54" s="11" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="T54" s="3" t="s">
-        <v>412</v>
+        <v>405</v>
       </c>
       <c r="U54" s="3" t="s">
-        <v>388</v>
+        <v>381</v>
       </c>
     </row>
     <row r="55" spans="1:21" ht="51.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="B55" s="45" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="C55" s="50" t="s">
         <v>60</v>
@@ -5393,10 +5425,10 @@
         <v>31</v>
       </c>
       <c r="E55" s="25" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G55" s="3"/>
       <c r="H55" s="151"/>
@@ -5414,21 +5446,21 @@
         <v>0</v>
       </c>
       <c r="S55" s="3" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="T55" s="3" t="s">
-        <v>411</v>
+        <v>404</v>
       </c>
       <c r="U55" s="3" t="s">
-        <v>390</v>
+        <v>383</v>
       </c>
     </row>
     <row r="56" spans="1:21" ht="57.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A56" s="14" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="B56" s="45" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="C56" s="50" t="s">
         <v>60</v>
@@ -5437,10 +5469,10 @@
         <v>31</v>
       </c>
       <c r="E56" s="25" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G56" s="3"/>
       <c r="H56" s="151"/>
@@ -5458,13 +5490,13 @@
         <v>0</v>
       </c>
       <c r="S56" s="3" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="T56" s="3" t="s">
-        <v>410</v>
+        <v>403</v>
       </c>
       <c r="U56" s="3" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
     </row>
     <row r="57" spans="1:21" ht="14.25" x14ac:dyDescent="0.2">
@@ -5492,7 +5524,7 @@
     </row>
     <row r="58" spans="1:21" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A58" s="172" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="B58" s="173"/>
       <c r="C58" s="173"/>
@@ -5517,10 +5549,10 @@
     </row>
     <row r="59" spans="1:21" ht="91.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A59" s="17" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="B59" s="51" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="C59" s="38" t="s">
         <v>21</v>
@@ -5529,60 +5561,60 @@
         <v>22</v>
       </c>
       <c r="E59" s="28" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G59" s="3"/>
       <c r="H59" s="160" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="I59" s="51" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="J59" s="51"/>
       <c r="K59" s="51" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="L59" s="51" t="s">
+        <v>311</v>
+      </c>
+      <c r="M59" s="51" t="s">
+        <v>312</v>
+      </c>
+      <c r="N59" s="51" t="s">
+        <v>313</v>
+      </c>
+      <c r="O59" s="51" t="s">
+        <v>314</v>
+      </c>
+      <c r="P59" s="51" t="s">
+        <v>315</v>
+      </c>
+      <c r="Q59" s="51" t="s">
         <v>316</v>
-      </c>
-      <c r="M59" s="51" t="s">
-        <v>317</v>
-      </c>
-      <c r="N59" s="51" t="s">
-        <v>318</v>
-      </c>
-      <c r="O59" s="51" t="s">
-        <v>319</v>
-      </c>
-      <c r="P59" s="51" t="s">
-        <v>320</v>
-      </c>
-      <c r="Q59" s="51" t="s">
-        <v>321</v>
       </c>
       <c r="R59" s="161">
         <f t="shared" ref="R59:R68" si="4">COUNTA(H59:Q59)/10</f>
         <v>0.9</v>
       </c>
       <c r="S59" s="3" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="T59" s="3" t="s">
-        <v>409</v>
+        <v>402</v>
       </c>
       <c r="U59" s="3" t="s">
-        <v>392</v>
+        <v>385</v>
       </c>
     </row>
     <row r="60" spans="1:21" ht="57.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A60" s="17" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="B60" s="51" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="C60" s="52" t="s">
         <v>21</v>
@@ -5591,10 +5623,10 @@
         <v>22</v>
       </c>
       <c r="E60" s="28" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G60" s="3"/>
       <c r="H60" s="160"/>
@@ -5603,14 +5635,14 @@
       <c r="K60" s="51"/>
       <c r="L60" s="51"/>
       <c r="M60" s="51" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="N60" s="51" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="O60" s="51"/>
       <c r="P60" s="51" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="Q60" s="51"/>
       <c r="R60" s="161">
@@ -5618,33 +5650,33 @@
         <v>0.3</v>
       </c>
       <c r="S60" s="3" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="T60" s="3" t="s">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="U60" s="3" t="s">
-        <v>393</v>
+        <v>386</v>
       </c>
     </row>
     <row r="61" spans="1:21" ht="43.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A61" s="17" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="B61" s="51" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="C61" s="38" t="s">
         <v>21</v>
       </c>
       <c r="D61" s="51" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="E61" s="28" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G61" s="3"/>
       <c r="H61" s="160"/>
@@ -5662,21 +5694,21 @@
         <v>0</v>
       </c>
       <c r="S61" s="3" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="T61" s="3" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="U61" s="3" t="s">
-        <v>394</v>
+        <v>387</v>
       </c>
     </row>
     <row r="62" spans="1:21" ht="43.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A62" s="18" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="B62" s="53" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="C62" s="54" t="s">
         <v>60</v>
@@ -5685,10 +5717,10 @@
         <v>22</v>
       </c>
       <c r="E62" s="29" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G62" s="3"/>
       <c r="H62" s="162"/>
@@ -5706,21 +5738,21 @@
         <v>0</v>
       </c>
       <c r="S62" s="3" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="T62" s="3" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="U62" s="3" t="s">
-        <v>395</v>
+        <v>388</v>
       </c>
     </row>
     <row r="63" spans="1:21" ht="43.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A63" s="18" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="B63" s="53" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="C63" s="54" t="s">
         <v>60</v>
@@ -5729,10 +5761,10 @@
         <v>22</v>
       </c>
       <c r="E63" s="29" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G63" s="3"/>
       <c r="H63" s="162"/>
@@ -5750,87 +5782,87 @@
         <v>0</v>
       </c>
       <c r="S63" s="3" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="T63" s="3" t="s">
-        <v>407</v>
+        <v>400</v>
       </c>
       <c r="U63" s="3" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
     </row>
     <row r="64" spans="1:21" ht="114.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A64" s="18" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="B64" s="53" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="C64" s="54" t="s">
         <v>60</v>
       </c>
       <c r="D64" s="53" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="E64" s="29" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G64" s="3"/>
       <c r="H64" s="162"/>
       <c r="I64" s="53" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="J64" s="53" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="K64" s="53" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="L64" s="53" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="M64" s="53"/>
       <c r="N64" s="53"/>
       <c r="O64" s="53"/>
       <c r="P64" s="53"/>
       <c r="Q64" s="53" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="R64" s="163">
         <f t="shared" si="4"/>
         <v>0.5</v>
       </c>
       <c r="S64" s="3" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="T64" s="3" t="s">
-        <v>403</v>
+        <v>396</v>
       </c>
       <c r="U64" s="3" t="s">
-        <v>397</v>
+        <v>390</v>
       </c>
     </row>
     <row r="65" spans="1:21" ht="39" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A65" s="18" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
       <c r="B65" s="53" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="C65" s="54" t="s">
         <v>60</v>
       </c>
       <c r="D65" s="53" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E65" s="29" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G65" s="3"/>
       <c r="H65" s="162"/>
@@ -5848,19 +5880,19 @@
         <v>0</v>
       </c>
       <c r="S65" s="3" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="T65" s="3"/>
       <c r="U65" s="3" t="s">
-        <v>398</v>
+        <v>391</v>
       </c>
     </row>
     <row r="66" spans="1:21" ht="72" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A66" s="18" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="B66" s="53" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
       <c r="C66" s="54" t="s">
         <v>60</v>
@@ -5869,10 +5901,10 @@
         <v>22</v>
       </c>
       <c r="E66" s="29" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="F66" s="8" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G66" s="8"/>
       <c r="H66" s="162"/>
@@ -5890,21 +5922,21 @@
         <v>0</v>
       </c>
       <c r="S66" s="3" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="T66" s="3" t="s">
-        <v>404</v>
+        <v>397</v>
       </c>
       <c r="U66" s="3" t="s">
-        <v>400</v>
+        <v>393</v>
       </c>
     </row>
     <row r="67" spans="1:21" ht="57.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A67" s="18" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="B67" s="53" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="C67" s="54" t="s">
         <v>60</v>
@@ -5913,10 +5945,10 @@
         <v>22</v>
       </c>
       <c r="E67" s="29" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="F67" s="8" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G67" s="8"/>
       <c r="H67" s="162"/>
@@ -5934,21 +5966,21 @@
         <v>0</v>
       </c>
       <c r="S67" s="3" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="T67" s="9" t="s">
-        <v>405</v>
+        <v>398</v>
       </c>
       <c r="U67" s="3" t="s">
-        <v>401</v>
+        <v>394</v>
       </c>
     </row>
     <row r="68" spans="1:21" ht="43.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A68" s="18" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="B68" s="53" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="C68" s="54" t="s">
         <v>60</v>
@@ -5957,10 +5989,10 @@
         <v>22</v>
       </c>
       <c r="E68" s="29" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="F68" s="8" t="s">
-        <v>201</v>
+        <v>452</v>
       </c>
       <c r="G68" s="8"/>
       <c r="H68" s="162"/>
@@ -5978,13 +6010,13 @@
         <v>0</v>
       </c>
       <c r="S68" s="3" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="T68" s="9" t="s">
-        <v>406</v>
+        <v>399</v>
       </c>
       <c r="U68" s="3" t="s">
-        <v>402</v>
+        <v>395</v>
       </c>
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.2">
@@ -6012,10 +6044,10 @@
     </row>
     <row r="70" spans="1:21" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A70" s="10" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B70" s="56" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="C70" s="57" t="s">
         <v>60</v>
@@ -6038,13 +6070,13 @@
       <c r="Q70" s="166"/>
       <c r="R70" s="114"/>
       <c r="S70" s="3" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="T70" s="3" t="s">
-        <v>389</v>
+        <v>382</v>
       </c>
       <c r="U70" s="3" t="s">
-        <v>399</v>
+        <v>392</v>
       </c>
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Regenerate empaTAPP catalog and constrain analyteColumns to it
Reshapes 26 analyteColumns/*.json catalog files to the hybrid
JSON Schema + examples annotation form, regenerates schema.yaml with
the oneOf constraint over them, and aligns exampleempaTAPP-all.json's
analyte-column entries to use each catalog file's canonical instance
(prior hand-authored entries used schema:inDefinedTermSet as a plain
URI string and a few off-by-a-word schema:name values that the new
const constraints reject).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TAPP_EPMA_filled.xlsx
+++ b/docs/TAPP_EPMA_filled.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/944a82e2ddcde9eb/Documents/GithubC/USGIN/geochemBuildingBlocks/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="299" documentId="11_3C209AD99577444EEF615C96566D1EBF266D99FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F1E778BF-00DE-4010-B5A4-4CECD611067F}"/>
+  <xr:revisionPtr revIDLastSave="301" documentId="11_3C209AD99577444EEF615C96566D1EBF266D99FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E128C9A9-D278-4B17-86BE-75B69BB4BEA7}"/>
   <bookViews>
-    <workbookView xWindow="8520" yWindow="990" windowWidth="27930" windowHeight="14610" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1245" yWindow="8535" windowWidth="27930" windowHeight="14610" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TAPP" sheetId="1" r:id="rId1"/>
@@ -964,9 +964,6 @@
     <t>Method (e.g., single-sample mean) + blank material name</t>
   </si>
   <si>
-    <t>Match. Method-level parameter with free-text schema:description; alternatively a Data Processing step's description.</t>
-  </si>
-  <si>
     <t>Normalization / Standards-Based Correction</t>
   </si>
   <si>
@@ -986,9 +983,6 @@
   </si>
   <si>
     <t>e.g., 10-12 %</t>
-  </si>
-  <si>
-    <t>Match. Method-level parameter with ada:dataType='number', schema:unitText='%'.</t>
   </si>
   <si>
     <t>Background Correction Method</t>
@@ -1609,6 +1603,12 @@
 silica glass, 
 coesite aggregates, 
 mesostasis</t>
+  </si>
+  <si>
+    <t>Match. Method-level parameter</t>
+  </si>
+  <si>
+    <t>Match. Method-level parameter with free-text schema:description</t>
   </si>
 </sst>
 </file>
@@ -2954,7 +2954,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="G1" s="2"/>
       <c r="H1" s="112" t="s">
@@ -2997,7 +2997,7 @@
         <v>17</v>
       </c>
       <c r="U1" s="3" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.2">
@@ -3078,10 +3078,10 @@
         <v>1</v>
       </c>
       <c r="S3" s="63" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="T3" s="169" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="U3" s="63"/>
     </row>
@@ -3138,13 +3138,13 @@
         <v>1</v>
       </c>
       <c r="S4" s="69" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="T4" s="170" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="U4" s="69" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="5" spans="1:21" s="70" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
@@ -3200,14 +3200,14 @@
         <v>1</v>
       </c>
       <c r="S5" s="69" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="T5" s="170" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="U5" s="69"/>
     </row>
-    <row r="6" spans="1:21" s="70" customFormat="1" ht="42.75" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:21" s="70" customFormat="1" ht="57" x14ac:dyDescent="0.2">
       <c r="A6" s="65" t="s">
         <v>46</v>
       </c>
@@ -3260,10 +3260,10 @@
         <v>1</v>
       </c>
       <c r="S6" s="69" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="T6" s="170" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="U6" s="69"/>
     </row>
@@ -3300,10 +3300,10 @@
         <v>0</v>
       </c>
       <c r="S7" s="69" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="T7" s="170" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="U7" s="69"/>
     </row>
@@ -3340,10 +3340,10 @@
         <v>0</v>
       </c>
       <c r="S8" s="69" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="T8" s="170" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="U8" s="69"/>
     </row>
@@ -3380,13 +3380,13 @@
         <v>0</v>
       </c>
       <c r="S9" s="69" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="T9" s="170" t="s">
+        <v>410</v>
+      </c>
+      <c r="U9" s="69" t="s">
         <v>412</v>
-      </c>
-      <c r="U9" s="69" t="s">
-        <v>414</v>
       </c>
     </row>
     <row r="10" spans="1:21" s="70" customFormat="1" ht="42.75" x14ac:dyDescent="0.2">
@@ -3422,10 +3422,10 @@
         <v>0</v>
       </c>
       <c r="S10" s="69" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="T10" s="170" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="U10" s="69"/>
     </row>
@@ -3499,7 +3499,7 @@
         <v>78</v>
       </c>
       <c r="I13" s="81" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="J13" s="81" t="s">
         <v>79</v>
@@ -3530,10 +3530,10 @@
         <v>1</v>
       </c>
       <c r="S13" s="69" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="T13" s="69" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="U13" s="69"/>
     </row>
@@ -3590,13 +3590,13 @@
         <v>1</v>
       </c>
       <c r="S14" s="69" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="T14" s="69" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="U14" s="69" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="15" spans="1:21" s="70" customFormat="1" ht="14.25" x14ac:dyDescent="0.2">
@@ -3700,14 +3700,14 @@
         <v>1</v>
       </c>
       <c r="S17" s="69" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="T17" s="170" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="U17" s="69"/>
     </row>
-    <row r="18" spans="1:21" s="70" customFormat="1" ht="42.75" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:21" s="70" customFormat="1" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A18" s="88" t="s">
         <v>108</v>
       </c>
@@ -3760,10 +3760,10 @@
         <v>1</v>
       </c>
       <c r="S18" s="69" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="T18" s="170" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="U18" s="69"/>
     </row>
@@ -3804,14 +3804,14 @@
         <v>0.2</v>
       </c>
       <c r="S19" s="69" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="T19" s="69" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="U19" s="69"/>
     </row>
-    <row r="20" spans="1:21" s="70" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:21" s="70" customFormat="1" ht="57" x14ac:dyDescent="0.2">
       <c r="A20" s="88" t="s">
         <v>123</v>
       </c>
@@ -3852,13 +3852,13 @@
         <v>0.4</v>
       </c>
       <c r="S20" s="69" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="T20" s="170" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="U20" s="69" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
     <row r="21" spans="1:21" s="70" customFormat="1" ht="57" x14ac:dyDescent="0.2">
@@ -3906,13 +3906,13 @@
         <v>0.6</v>
       </c>
       <c r="S21" s="69" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="T21" s="170" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="U21" s="69" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
     </row>
     <row r="22" spans="1:21" s="70" customFormat="1" ht="57" x14ac:dyDescent="0.2">
@@ -3950,16 +3950,16 @@
         <v>0.1</v>
       </c>
       <c r="S22" s="69" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="T22" s="69" t="s">
         <v>140</v>
       </c>
       <c r="U22" s="69" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="23" spans="1:21" s="70" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="23" spans="1:21" s="70" customFormat="1" ht="57" x14ac:dyDescent="0.2">
       <c r="A23" s="92" t="s">
         <v>141</v>
       </c>
@@ -3994,13 +3994,13 @@
         <v>0.1</v>
       </c>
       <c r="S23" s="69" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="T23" s="69" t="s">
         <v>145</v>
       </c>
       <c r="U23" s="69" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
     <row r="24" spans="1:21" s="70" customFormat="1" ht="14.25" x14ac:dyDescent="0.2">
@@ -4104,13 +4104,13 @@
         <v>1</v>
       </c>
       <c r="S26" s="69" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="T26" s="170" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="U26" s="171" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
     </row>
     <row r="27" spans="1:21" s="70" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
@@ -4166,13 +4166,13 @@
         <v>1</v>
       </c>
       <c r="S27" s="101" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="T27" s="170" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="U27" s="171" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
     </row>
     <row r="28" spans="1:21" s="70" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
@@ -4226,13 +4226,13 @@
         <v>0.9</v>
       </c>
       <c r="S28" s="101" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="T28" s="170" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="U28" s="171" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
     </row>
     <row r="29" spans="1:21" s="70" customFormat="1" ht="51" x14ac:dyDescent="0.2">
@@ -4274,10 +4274,10 @@
         <v>179</v>
       </c>
       <c r="U29" s="69" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="30" spans="1:21" s="70" customFormat="1" ht="71.25" x14ac:dyDescent="0.2">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="30" spans="1:21" s="70" customFormat="1" ht="85.5" x14ac:dyDescent="0.2">
       <c r="A30" s="102" t="s">
         <v>180</v>
       </c>
@@ -4320,10 +4320,10 @@
         <v>186</v>
       </c>
       <c r="U30" s="69" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="31" spans="1:21" s="111" customFormat="1" ht="72" thickBot="1" x14ac:dyDescent="0.25">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="31" spans="1:21" s="111" customFormat="1" ht="100.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A31" s="106" t="s">
         <v>187</v>
       </c>
@@ -4362,7 +4362,7 @@
         <v>190</v>
       </c>
       <c r="U31" s="110" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="32" spans="1:21" ht="234" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -4403,10 +4403,10 @@
         <v>195</v>
       </c>
       <c r="T32" s="3" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="U32" s="3" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
     </row>
     <row r="33" spans="1:21" ht="77.25" thickBot="1" x14ac:dyDescent="0.25">
@@ -4426,7 +4426,7 @@
         <v>199</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G33" s="3"/>
       <c r="H33" s="143" t="s">
@@ -4436,7 +4436,7 @@
         <v>201</v>
       </c>
       <c r="J33" s="36" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="K33" s="36" t="s">
         <v>200</v>
@@ -4451,10 +4451,10 @@
         <v>203</v>
       </c>
       <c r="O33" s="36" t="s">
+        <v>457</v>
+      </c>
+      <c r="P33" s="36" t="s">
         <v>459</v>
-      </c>
-      <c r="P33" s="36" t="s">
-        <v>461</v>
       </c>
       <c r="Q33" s="36" t="s">
         <v>203</v>
@@ -4467,10 +4467,10 @@
         <v>163</v>
       </c>
       <c r="T33" s="3" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="U33" s="3" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="34" spans="1:21" ht="39" thickBot="1" x14ac:dyDescent="0.25">
@@ -4490,7 +4490,7 @@
         <v>206</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G34" s="3"/>
       <c r="H34" s="143" t="s">
@@ -4534,7 +4534,7 @@
         <v>209</v>
       </c>
       <c r="U34" s="3" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
     </row>
     <row r="35" spans="1:21" ht="39" thickBot="1" x14ac:dyDescent="0.25">
@@ -4554,7 +4554,7 @@
         <v>213</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G35" s="3"/>
       <c r="H35" s="145"/>
@@ -4578,7 +4578,7 @@
         <v>214</v>
       </c>
       <c r="U35" s="3" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="36" spans="1:21" ht="39" thickBot="1" x14ac:dyDescent="0.25">
@@ -4598,7 +4598,7 @@
         <v>213</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G36" s="3"/>
       <c r="H36" s="145"/>
@@ -4622,10 +4622,10 @@
         <v>217</v>
       </c>
       <c r="U36" s="3" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="37" spans="1:21" ht="72" thickBot="1" x14ac:dyDescent="0.25">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="37" spans="1:21" ht="86.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
         <v>218</v>
       </c>
@@ -4642,7 +4642,7 @@
         <v>220</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G37" s="3"/>
       <c r="H37" s="143"/>
@@ -4668,10 +4668,10 @@
         <v>222</v>
       </c>
       <c r="U37" s="3" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="38" spans="1:21" ht="64.5" thickBot="1" x14ac:dyDescent="0.25">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="38" spans="1:21" ht="57.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A38" s="13" t="s">
         <v>223</v>
       </c>
@@ -4688,7 +4688,7 @@
         <v>225</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G38" s="3"/>
       <c r="H38" s="145"/>
@@ -4712,7 +4712,7 @@
         <v>226</v>
       </c>
       <c r="U38" s="3" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="39" spans="1:21" ht="39" thickBot="1" x14ac:dyDescent="0.25">
@@ -4732,7 +4732,7 @@
         <v>229</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G39" s="3"/>
       <c r="H39" s="145"/>
@@ -4756,7 +4756,7 @@
         <v>230</v>
       </c>
       <c r="U39" s="3" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="40" spans="1:21" ht="129" thickBot="1" x14ac:dyDescent="0.25">
@@ -4776,16 +4776,16 @@
         <v>233</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G40" s="3"/>
       <c r="H40" s="143" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="I40" s="36"/>
       <c r="J40" s="36"/>
       <c r="K40" s="36" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="L40" s="36"/>
       <c r="M40" s="36"/>
@@ -4804,7 +4804,7 @@
         <v>236</v>
       </c>
       <c r="U40" s="3" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
     </row>
     <row r="41" spans="1:21" ht="57.75" thickBot="1" x14ac:dyDescent="0.25">
@@ -4824,7 +4824,7 @@
         <v>240</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G41" s="3"/>
       <c r="H41" s="143" t="s">
@@ -4858,7 +4858,7 @@
         <v>245</v>
       </c>
       <c r="U41" s="3" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="42" spans="1:21" ht="57.75" thickBot="1" x14ac:dyDescent="0.25">
@@ -4878,7 +4878,7 @@
         <v>248</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G42" s="3"/>
       <c r="H42" s="143" t="s">
@@ -4910,7 +4910,7 @@
         <v>251</v>
       </c>
       <c r="U42" s="3" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
     <row r="43" spans="1:21" ht="72" thickBot="1" x14ac:dyDescent="0.25">
@@ -4930,7 +4930,7 @@
         <v>255</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G43" s="3"/>
       <c r="H43" s="145"/>
@@ -4954,7 +4954,7 @@
         <v>256</v>
       </c>
       <c r="U43" s="3" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="44" spans="1:21" ht="14.25" x14ac:dyDescent="0.2">
@@ -5005,7 +5005,7 @@
       <c r="T45" s="3"/>
       <c r="U45" s="3"/>
     </row>
-    <row r="46" spans="1:21" ht="114" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:21" ht="142.5" x14ac:dyDescent="0.2">
       <c r="A46" s="6" t="s">
         <v>258</v>
       </c>
@@ -5052,16 +5052,16 @@
         <v>0.7</v>
       </c>
       <c r="S46" s="11" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="T46" s="3" t="s">
         <v>264</v>
       </c>
       <c r="U46" s="3" t="s">
-        <v>445</v>
-      </c>
-    </row>
-    <row r="47" spans="1:21" ht="51" x14ac:dyDescent="0.2">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="47" spans="1:21" ht="57" x14ac:dyDescent="0.2">
       <c r="A47" s="6" t="s">
         <v>265</v>
       </c>
@@ -5100,7 +5100,7 @@
         <v>268</v>
       </c>
       <c r="U47" s="3" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="48" spans="1:21" ht="57" x14ac:dyDescent="0.2">
@@ -5146,10 +5146,10 @@
         <v>275</v>
       </c>
       <c r="U48" s="3" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="49" spans="1:21" ht="99.75" x14ac:dyDescent="0.2">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="49" spans="1:21" ht="128.25" x14ac:dyDescent="0.2">
       <c r="A49" s="6" t="s">
         <v>276</v>
       </c>
@@ -5188,10 +5188,10 @@
         <v>279</v>
       </c>
       <c r="U49" s="3" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="50" spans="1:21" ht="64.5" thickBot="1" x14ac:dyDescent="0.25">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="50" spans="1:21" ht="57.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A50" s="7" t="s">
         <v>280</v>
       </c>
@@ -5230,7 +5230,7 @@
         <v>283</v>
       </c>
       <c r="U50" s="3" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="51" spans="1:21" ht="43.5" thickBot="1" x14ac:dyDescent="0.25">
@@ -5250,7 +5250,7 @@
         <v>286</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G51" s="3"/>
       <c r="H51" s="151"/>
@@ -5271,18 +5271,18 @@
         <v>208</v>
       </c>
       <c r="T51" s="3" t="s">
-        <v>287</v>
+        <v>462</v>
       </c>
       <c r="U51" s="3" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="52" spans="1:21" ht="43.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
+        <v>287</v>
+      </c>
+      <c r="B52" s="45" t="s">
         <v>288</v>
-      </c>
-      <c r="B52" s="45" t="s">
-        <v>289</v>
       </c>
       <c r="C52" s="46" t="s">
         <v>60</v>
@@ -5291,10 +5291,10 @@
         <v>22</v>
       </c>
       <c r="E52" s="25" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G52" s="3"/>
       <c r="H52" s="151"/>
@@ -5315,18 +5315,18 @@
         <v>208</v>
       </c>
       <c r="T52" s="3" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="U52" s="3" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="53" spans="1:21" ht="39" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A53" s="15" t="s">
+        <v>291</v>
+      </c>
+      <c r="B53" s="47" t="s">
         <v>292</v>
-      </c>
-      <c r="B53" s="47" t="s">
-        <v>293</v>
       </c>
       <c r="C53" s="48" t="s">
         <v>60</v>
@@ -5335,10 +5335,10 @@
         <v>22</v>
       </c>
       <c r="E53" s="26" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G53" s="3"/>
       <c r="H53" s="153"/>
@@ -5359,18 +5359,18 @@
         <v>208</v>
       </c>
       <c r="T53" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="U53" s="3" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="54" spans="1:21" ht="143.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="16" t="s">
+        <v>294</v>
+      </c>
+      <c r="B54" s="49" t="s">
         <v>295</v>
-      </c>
-      <c r="U53" s="3" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="54" spans="1:21" ht="114.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="16" t="s">
-        <v>296</v>
-      </c>
-      <c r="B54" s="49" t="s">
-        <v>297</v>
       </c>
       <c r="C54" s="38" t="s">
         <v>21</v>
@@ -5379,10 +5379,10 @@
         <v>31</v>
       </c>
       <c r="E54" s="27" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G54" s="3"/>
       <c r="H54" s="155"/>
@@ -5391,7 +5391,7 @@
       <c r="K54" s="49"/>
       <c r="L54" s="49"/>
       <c r="M54" s="49" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="N54" s="49"/>
       <c r="O54" s="49"/>
@@ -5405,18 +5405,18 @@
         <v>208</v>
       </c>
       <c r="T54" s="3" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="U54" s="3" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
     </row>
     <row r="55" spans="1:21" ht="51.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B55" s="45" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C55" s="50" t="s">
         <v>60</v>
@@ -5425,10 +5425,10 @@
         <v>31</v>
       </c>
       <c r="E55" s="25" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G55" s="3"/>
       <c r="H55" s="151"/>
@@ -5449,18 +5449,18 @@
         <v>208</v>
       </c>
       <c r="T55" s="3" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="U55" s="3" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="56" spans="1:21" ht="57.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A56" s="14" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="B56" s="45" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C56" s="50" t="s">
         <v>60</v>
@@ -5469,10 +5469,10 @@
         <v>31</v>
       </c>
       <c r="E56" s="25" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G56" s="3"/>
       <c r="H56" s="151"/>
@@ -5493,10 +5493,10 @@
         <v>208</v>
       </c>
       <c r="T56" s="3" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="U56" s="3" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
     </row>
     <row r="57" spans="1:21" ht="14.25" x14ac:dyDescent="0.2">
@@ -5524,7 +5524,7 @@
     </row>
     <row r="58" spans="1:21" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A58" s="172" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B58" s="173"/>
       <c r="C58" s="173"/>
@@ -5549,10 +5549,10 @@
     </row>
     <row r="59" spans="1:21" ht="91.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A59" s="17" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="B59" s="51" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C59" s="38" t="s">
         <v>21</v>
@@ -5561,39 +5561,39 @@
         <v>22</v>
       </c>
       <c r="E59" s="28" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G59" s="3"/>
       <c r="H59" s="160" t="s">
         <v>234</v>
       </c>
       <c r="I59" s="51" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="J59" s="51"/>
       <c r="K59" s="51" t="s">
         <v>235</v>
       </c>
       <c r="L59" s="51" t="s">
+        <v>309</v>
+      </c>
+      <c r="M59" s="51" t="s">
+        <v>310</v>
+      </c>
+      <c r="N59" s="51" t="s">
         <v>311</v>
       </c>
-      <c r="M59" s="51" t="s">
+      <c r="O59" s="51" t="s">
         <v>312</v>
       </c>
-      <c r="N59" s="51" t="s">
+      <c r="P59" s="51" t="s">
         <v>313</v>
       </c>
-      <c r="O59" s="51" t="s">
+      <c r="Q59" s="51" t="s">
         <v>314</v>
-      </c>
-      <c r="P59" s="51" t="s">
-        <v>315</v>
-      </c>
-      <c r="Q59" s="51" t="s">
-        <v>316</v>
       </c>
       <c r="R59" s="161">
         <f t="shared" ref="R59:R68" si="4">COUNTA(H59:Q59)/10</f>
@@ -5603,18 +5603,18 @@
         <v>208</v>
       </c>
       <c r="T59" s="3" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="U59" s="3" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="60" spans="1:21" ht="57.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A60" s="17" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B60" s="51" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="C60" s="52" t="s">
         <v>21</v>
@@ -5623,10 +5623,10 @@
         <v>22</v>
       </c>
       <c r="E60" s="28" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G60" s="3"/>
       <c r="H60" s="160"/>
@@ -5635,14 +5635,14 @@
       <c r="K60" s="51"/>
       <c r="L60" s="51"/>
       <c r="M60" s="51" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="N60" s="51" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="O60" s="51"/>
       <c r="P60" s="51" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="Q60" s="51"/>
       <c r="R60" s="161">
@@ -5653,18 +5653,18 @@
         <v>208</v>
       </c>
       <c r="T60" s="3" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="U60" s="3" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="61" spans="1:21" ht="43.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A61" s="17" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="B61" s="51" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C61" s="38" t="s">
         <v>21</v>
@@ -5673,10 +5673,10 @@
         <v>271</v>
       </c>
       <c r="E61" s="28" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G61" s="3"/>
       <c r="H61" s="160"/>
@@ -5697,18 +5697,18 @@
         <v>208</v>
       </c>
       <c r="T61" s="3" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="U61" s="3" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="62" spans="1:21" ht="43.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A62" s="18" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="B62" s="53" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="C62" s="54" t="s">
         <v>60</v>
@@ -5717,10 +5717,10 @@
         <v>22</v>
       </c>
       <c r="E62" s="29" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G62" s="3"/>
       <c r="H62" s="162"/>
@@ -5741,18 +5741,18 @@
         <v>208</v>
       </c>
       <c r="T62" s="3" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="U62" s="3" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="63" spans="1:21" ht="43.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A63" s="18" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="B63" s="53" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="C63" s="54" t="s">
         <v>60</v>
@@ -5761,10 +5761,10 @@
         <v>22</v>
       </c>
       <c r="E63" s="29" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G63" s="3"/>
       <c r="H63" s="162"/>
@@ -5785,51 +5785,51 @@
         <v>208</v>
       </c>
       <c r="T63" s="3" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="U63" s="3" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="64" spans="1:21" ht="114.75" thickBot="1" x14ac:dyDescent="0.25">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="64" spans="1:21" ht="171.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A64" s="18" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="B64" s="53" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C64" s="54" t="s">
         <v>60</v>
       </c>
       <c r="D64" s="53" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="E64" s="29" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G64" s="3"/>
       <c r="H64" s="162"/>
       <c r="I64" s="53" t="s">
+        <v>336</v>
+      </c>
+      <c r="J64" s="53" t="s">
+        <v>337</v>
+      </c>
+      <c r="K64" s="53" t="s">
         <v>338</v>
       </c>
-      <c r="J64" s="53" t="s">
+      <c r="L64" s="53" t="s">
         <v>339</v>
-      </c>
-      <c r="K64" s="53" t="s">
-        <v>340</v>
-      </c>
-      <c r="L64" s="53" t="s">
-        <v>341</v>
       </c>
       <c r="M64" s="53"/>
       <c r="N64" s="53"/>
       <c r="O64" s="53"/>
       <c r="P64" s="53"/>
       <c r="Q64" s="53" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="R64" s="163">
         <f t="shared" si="4"/>
@@ -5839,18 +5839,18 @@
         <v>208</v>
       </c>
       <c r="T64" s="3" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="U64" s="3" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="65" spans="1:21" ht="39" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A65" s="18" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="B65" s="53" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C65" s="54" t="s">
         <v>60</v>
@@ -5859,10 +5859,10 @@
         <v>130</v>
       </c>
       <c r="E65" s="29" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G65" s="3"/>
       <c r="H65" s="162"/>
@@ -5884,15 +5884,15 @@
       </c>
       <c r="T65" s="3"/>
       <c r="U65" s="3" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
     <row r="66" spans="1:21" ht="72" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A66" s="18" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B66" s="53" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="C66" s="54" t="s">
         <v>60</v>
@@ -5901,10 +5901,10 @@
         <v>22</v>
       </c>
       <c r="E66" s="29" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="F66" s="8" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G66" s="8"/>
       <c r="H66" s="162"/>
@@ -5925,18 +5925,18 @@
         <v>208</v>
       </c>
       <c r="T66" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="U66" s="3" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
     </row>
     <row r="67" spans="1:21" ht="57.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A67" s="18" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="B67" s="53" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="C67" s="54" t="s">
         <v>60</v>
@@ -5945,10 +5945,10 @@
         <v>22</v>
       </c>
       <c r="E67" s="29" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="F67" s="8" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G67" s="8"/>
       <c r="H67" s="162"/>
@@ -5969,18 +5969,18 @@
         <v>208</v>
       </c>
       <c r="T67" s="9" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="U67" s="3" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="68" spans="1:21" ht="43.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A68" s="18" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B68" s="53" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="C68" s="54" t="s">
         <v>60</v>
@@ -5989,10 +5989,10 @@
         <v>22</v>
       </c>
       <c r="E68" s="29" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="F68" s="8" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G68" s="8"/>
       <c r="H68" s="162"/>
@@ -6013,10 +6013,10 @@
         <v>208</v>
       </c>
       <c r="T68" s="9" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="U68" s="3" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.2">
@@ -6044,10 +6044,10 @@
     </row>
     <row r="70" spans="1:21" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A70" s="10" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="B70" s="56" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="C70" s="57" t="s">
         <v>60</v>
@@ -6070,13 +6070,13 @@
       <c r="Q70" s="166"/>
       <c r="R70" s="114"/>
       <c r="S70" s="3" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="T70" s="3" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="U70" s="3" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.2">

</xml_diff>